<commit_message>
Expand validation example to 96-well plate
</commit_message>
<xml_diff>
--- a/example_2/data/validation_plate_0.xlsx
+++ b/example_2/data/validation_plate_0.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,6 +454,46 @@
           <t>4</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -465,13 +505,37 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="F2" t="n">
+        <v>9</v>
+      </c>
+      <c r="G2" t="n">
+        <v>11</v>
+      </c>
+      <c r="H2" t="n">
+        <v>13</v>
+      </c>
+      <c r="I2" t="n">
+        <v>15</v>
+      </c>
+      <c r="J2" t="n">
+        <v>17</v>
+      </c>
+      <c r="K2" t="n">
+        <v>19</v>
+      </c>
+      <c r="L2" t="n">
+        <v>21</v>
+      </c>
+      <c r="M2" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="3">
@@ -484,13 +548,37 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="F3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G3" t="n">
+        <v>12</v>
+      </c>
+      <c r="H3" t="n">
+        <v>14</v>
+      </c>
+      <c r="I3" t="n">
+        <v>16</v>
+      </c>
+      <c r="J3" t="n">
+        <v>18</v>
+      </c>
+      <c r="K3" t="n">
+        <v>20</v>
+      </c>
+      <c r="L3" t="n">
+        <v>22</v>
+      </c>
+      <c r="M3" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -503,13 +591,37 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E4" t="n">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="F4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G4" t="n">
+        <v>13</v>
+      </c>
+      <c r="H4" t="n">
+        <v>15</v>
+      </c>
+      <c r="I4" t="n">
+        <v>17</v>
+      </c>
+      <c r="J4" t="n">
+        <v>19</v>
+      </c>
+      <c r="K4" t="n">
+        <v>21</v>
+      </c>
+      <c r="L4" t="n">
+        <v>23</v>
+      </c>
+      <c r="M4" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -522,13 +634,209 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D5" t="n">
+        <v>8</v>
+      </c>
+      <c r="E5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" t="n">
+        <v>12</v>
+      </c>
+      <c r="G5" t="n">
+        <v>14</v>
+      </c>
+      <c r="H5" t="n">
+        <v>16</v>
+      </c>
+      <c r="I5" t="n">
+        <v>18</v>
+      </c>
+      <c r="J5" t="n">
+        <v>20</v>
+      </c>
+      <c r="K5" t="n">
+        <v>22</v>
+      </c>
+      <c r="L5" t="n">
+        <v>24</v>
+      </c>
+      <c r="M5" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>5</v>
       </c>
-      <c r="D5" t="n">
+      <c r="C6" t="n">
         <v>7</v>
       </c>
-      <c r="E5" t="n">
+      <c r="D6" t="n">
+        <v>9</v>
+      </c>
+      <c r="E6" t="n">
+        <v>11</v>
+      </c>
+      <c r="F6" t="n">
+        <v>13</v>
+      </c>
+      <c r="G6" t="n">
+        <v>15</v>
+      </c>
+      <c r="H6" t="n">
+        <v>17</v>
+      </c>
+      <c r="I6" t="n">
+        <v>19</v>
+      </c>
+      <c r="J6" t="n">
+        <v>21</v>
+      </c>
+      <c r="K6" t="n">
+        <v>23</v>
+      </c>
+      <c r="L6" t="n">
+        <v>25</v>
+      </c>
+      <c r="M6" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="n">
         <v>8</v>
+      </c>
+      <c r="D7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" t="n">
+        <v>12</v>
+      </c>
+      <c r="F7" t="n">
+        <v>14</v>
+      </c>
+      <c r="G7" t="n">
+        <v>16</v>
+      </c>
+      <c r="H7" t="n">
+        <v>18</v>
+      </c>
+      <c r="I7" t="n">
+        <v>20</v>
+      </c>
+      <c r="J7" t="n">
+        <v>22</v>
+      </c>
+      <c r="K7" t="n">
+        <v>24</v>
+      </c>
+      <c r="L7" t="n">
+        <v>26</v>
+      </c>
+      <c r="M7" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="n">
+        <v>9</v>
+      </c>
+      <c r="D8" t="n">
+        <v>11</v>
+      </c>
+      <c r="E8" t="n">
+        <v>13</v>
+      </c>
+      <c r="F8" t="n">
+        <v>15</v>
+      </c>
+      <c r="G8" t="n">
+        <v>17</v>
+      </c>
+      <c r="H8" t="n">
+        <v>19</v>
+      </c>
+      <c r="I8" t="n">
+        <v>21</v>
+      </c>
+      <c r="J8" t="n">
+        <v>23</v>
+      </c>
+      <c r="K8" t="n">
+        <v>25</v>
+      </c>
+      <c r="L8" t="n">
+        <v>27</v>
+      </c>
+      <c r="M8" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C9" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" t="n">
+        <v>12</v>
+      </c>
+      <c r="E9" t="n">
+        <v>14</v>
+      </c>
+      <c r="F9" t="n">
+        <v>16</v>
+      </c>
+      <c r="G9" t="n">
+        <v>18</v>
+      </c>
+      <c r="H9" t="n">
+        <v>20</v>
+      </c>
+      <c r="I9" t="n">
+        <v>22</v>
+      </c>
+      <c r="J9" t="n">
+        <v>24</v>
+      </c>
+      <c r="K9" t="n">
+        <v>26</v>
+      </c>
+      <c r="L9" t="n">
+        <v>28</v>
+      </c>
+      <c r="M9" t="n">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>